<commit_message>
Clarify PnP extra part quantities and tape purchasing guidance
</commit_message>
<xml_diff>
--- a/engineering/Osiris_PDB_REV1.1_XT60_Procurement_PnP.xlsx
+++ b/engineering/Osiris_PDB_REV1.1_XT60_Procurement_PnP.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="1" r:id="R9e21bc6bba3c4cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="2" r:id="R84b1294069aa4d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="1" r:id="R06626cba86694761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="2" r:id="Rf46dc1ceec2b436f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2069,7 +2069,7 @@
       <x:c r="N2" s="147"/>
       <x:c r="O2" s="142"/>
       <x:c r="P2" s="182" t="str">
-        <x:v>PnP purchasing guidance — October 7, 2026</x:v>
+        <x:v>PnP extra parts and purchasing guidance</x:v>
       </x:c>
       <x:c r="Q2" s="182"/>
       <x:c r="R2" s="182"/>
@@ -2081,7 +2081,7 @@
       <x:c r="X2" s="142"/>
       <x:c r="Y2" s="142"/>
     </x:row>
-    <x:row r="3" ht="23" hidden="0" customHeight="1">
+    <x:row r="3" ht="36" hidden="0" customHeight="1">
       <x:c r="A3" s="124"/>
       <x:c r="B3" s="124"/>
       <x:c r="C3" s="124"/>
@@ -2098,7 +2098,7 @@
       <x:c r="N3" s="124"/>
       <x:c r="O3" s="142"/>
       <x:c r="P3" s="182" t="str">
-        <x:v>Passives: MAX(100, 10 × required qty). All other parts: +20%, rounded up.</x:v>
+        <x:v>Passives: buy at least 100 pieces or 10 times required quantity, whichever is greater. Other parts: 20% extra, rounded up.</x:v>
       </x:c>
       <x:c r="Q3" s="182"/>
       <x:c r="R3" s="182"/>
@@ -2110,7 +2110,7 @@
       <x:c r="X3" s="142"/>
       <x:c r="Y3" s="142"/>
     </x:row>
-    <x:row r="4" ht="23" hidden="0" customHeight="1">
+    <x:row r="4" ht="36" hidden="0" customHeight="1">
       <x:c r="A4" s="152" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -2151,7 +2151,7 @@
       </x:c>
       <x:c r="O4" s="142"/>
       <x:c r="P4" s="182" t="str">
-        <x:v>Full reels preferred. Use Digi-Reel/equivalent extenders for small tape orders.</x:v>
+        <x:v>Buy the Final order qty in column R. Full reels preferred; ask for tape and cover-tape leaders/extenders for small tape orders.</x:v>
       </x:c>
       <x:c r="Q4" s="182"/>
       <x:c r="R4" s="182"/>
@@ -2163,7 +2163,7 @@
       <x:c r="X4" s="142"/>
       <x:c r="Y4" s="142"/>
     </x:row>
-    <x:row r="5" ht="23" hidden="0" customHeight="1">
+    <x:row r="5" ht="36" hidden="0" customHeight="1">
       <x:c r="A5" s="122"/>
       <x:c r="B5" s="122"/>
       <x:c r="C5" s="122"/>
@@ -2180,7 +2180,7 @@
       <x:c r="N5" s="122"/>
       <x:c r="O5" s="142"/>
       <x:c r="P5" s="182" t="str">
-        <x:v>Yellow override: round up for reel/MOQ. Recheck stock and prices at checkout.</x:v>
+        <x:v>Column Q accepts a larger order quantity for reels/MOQ. LCSC substitutions round up to supplier multiples. Recheck stock and prices.</x:v>
       </x:c>
       <x:c r="Q5" s="182"/>
       <x:c r="R5" s="182"/>
@@ -2472,7 +2472,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U10" s="175" t="str">
-        <x:v>Same value/package. 50 V, X7R, ±10%. C91185. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 50 V, X7R, ±10%. C91185. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V10" s="142"/>
       <x:c r="W10" s="175" t="str">
@@ -3017,7 +3017,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U17" s="142" t="str">
-        <x:v>Same value/package. 50 V, X7R, ±10%. C49678. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 50 V, X7R, ±10%. C49678. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V17" s="142"/>
       <x:c r="W17" s="142" t="str">
@@ -4032,7 +4032,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U30" s="175" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C26112. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C26112. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V30" s="142"/>
       <x:c r="W30" s="175" t="str">
@@ -4111,7 +4111,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U31" s="142" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17560. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17560. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V31" s="142"/>
       <x:c r="W31" s="142" t="str">
@@ -4269,7 +4269,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U33" s="142" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17797. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17797. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V33" s="142"/>
       <x:c r="W33" s="142" t="str">
@@ -4348,7 +4348,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U34" s="175" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17539. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17539. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V34" s="142"/>
       <x:c r="W34" s="175" t="str">
@@ -4427,7 +4427,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U35" s="142" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17415. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17415. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V35" s="142"/>
       <x:c r="W35" s="142" t="str">
@@ -4506,7 +4506,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U36" s="175" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17673. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17673. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V36" s="142"/>
       <x:c r="W36" s="175" t="str">
@@ -4664,7 +4664,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U38" s="175" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17513. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17513. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V38" s="142"/>
       <x:c r="W38" s="175" t="str">
@@ -4901,7 +4901,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U41" s="142" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17414. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17414. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V41" s="142"/>
       <x:c r="W41" s="142" t="str">
@@ -5138,7 +5138,7 @@
         <x:v>Passive: 100 or 10×</x:v>
       </x:c>
       <x:c r="U44" s="175" t="str">
-        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17408. Buy one lot per MPN.</x:v>
+        <x:v>Same value/package. 125 mW, 150 V, ±1%. C17408. Buy one lot per MPN. Full reel preferred; request tape/cover-tape leaders for small orders.</x:v>
       </x:c>
       <x:c r="V44" s="142"/>
       <x:c r="W44" s="175" t="str">
@@ -5793,51 +5793,51 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R76c4eb5c5ff6483e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R81979a57a56c4884"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R7e2ccdccf1b04ed2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="R124642d0a3844da9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Rd76556594ac543e7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="Rdd1a68474f474067"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="Rebd6e0e98dbd4336"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R90abf4e9b9d443e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="R64bb215ab5f94940"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="Rd86c4478d2b941a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R56817c8901ba4b39"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="R01ad1f6e7ad546aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="R953be8ac5da94529"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rf32481e53d8f4ca0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R33ad3461a7954a41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R0766df2c35fe47f8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R4eb9216660b749b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R555a4e7a4fff4c62"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="Rea557b12c3674683"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Rd079165abea74dac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="R24349fda03f047be"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="Rd6d45ddf1ab143d2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="R66380de57ee74659"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="R97d538dbdddb4008"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="R58ac4f9d333846f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R0d637c0eb98440f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R27287c34c35d4645"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R8f230643f06148d4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="Rac66d31d7e264373"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R018e89adbd264be7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="R49d72d5ca84244be"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R8a7259bc87a845c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="Rdb0804e759f645de"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="Rf5f129ac3f924b42"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="Rb4c32a9925614e2c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="R1e94658e592c42d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="Ra5711c258e4f4a3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="Rb7ceaf5371f44e18"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="R0f50258c88504357"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="Rba4191f514ab48dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="R786c49a32a2e4f49"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="R66908313314a4fb0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R425273b541f94699"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rc5b540feafae47cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R31df980a8fa34967"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="R4030aa2b09be416d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R577393089da548df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R9b6a23326a334715"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R23c0311105ad4544"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R2f12976fcb2c4ed7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="Re0f35bed6ece4653"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="R5ac792d241f742cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R95d9052cf16a484a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Ree913fd1c0164949"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="R770340699c274cd8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rf28e47914a714807"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R8776175fd86e41a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="Reada309ff92f41ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R29441d9e301a449f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R27fe07c573d5415b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="R3d0021d1f0084a9c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ra074ce5555e54b04"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="R4fca9ac153c64416"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="Rfb5dc83b01d544dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="R1f558779162d4473"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="Rac36460eda9b445b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="R869f7b4bc9584c94"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R2a92235a761e41e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Rb3a874beef32418e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Re42610016fd84b65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="Ra8cae8b1acc44c3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R78a4b473aae64110"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="Rfa2583ac44ff4768"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R4aa663d25242440b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="Rad9277ceda5f4df5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="Rf1a4804b8795489b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="Rfa66edb015d946c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="R190f97f3c5284130"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="Ra2ec0e497b184f4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="Re9f6faf1712e4d18"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="Rf2ce35d8168441ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="R277d598a932c4869"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="Rbf331e4579e84c5e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="Rad202e25e27a4220"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d202213244f44f1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb81a28acca44606"/>
 </x:worksheet>
 </file>
 

</xml_diff>